<commit_message>
fix: remove unfilled placeholder sources and dead SentinelOne feed URL
F6 Russia, Packetstorm, Secureworks were auto-detection failures that
never got real selectors, printing "config not filled in yet, skipping"
every run. Phylum and Veriti AI are already covered by the Veracode and
Check Point Exposure Management entries respectively. Removed all 5 from
config.json and the xlsx so auto-sync doesn't resurrect them.

Also fixed SentinelOne's feed URL (sentinelone.com/feed/ now 404s) to
the working sentinelone.com/blog/feed/.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CTI_Source_List.xlsx
+++ b/CTI_Source_List.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B222"/>
+  <dimension ref="A1:B217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="75" customWidth="1" style="4" min="1" max="1"/>
@@ -1864,1308 +1864,1248 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Packetstorm</t>
-        </is>
-      </c>
-      <c r="B114" s="7" t="inlineStr">
-        <is>
-          <t>https://packetstorm.news/</t>
+          <t>Praetorian</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://www.praetorian.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Praetorian</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>https://www.praetorian.com/blog/</t>
+          <t>PT Security</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>https://global.ptsecurity.com/analytics/pt-esc-threat-intelligence</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>PT Security</t>
-        </is>
-      </c>
-      <c r="B116" s="7" t="inlineStr">
-        <is>
-          <t>https://global.ptsecurity.com/analytics/pt-esc-threat-intelligence</t>
+          <t>Red Canary</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://redcanary.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Red Canary</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>https://redcanary.com/blog/</t>
+          <t>Sansec</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>https://sansec.io/research</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Sansec</t>
-        </is>
-      </c>
-      <c r="B118" s="7" t="inlineStr">
-        <is>
-          <t>https://sansec.io/research</t>
+          <t>Sweet Security</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.sweet.security/blog</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Sweet Security</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.sweet.security/blog</t>
+          <t>https://blog.cloudflare.com/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>DMPDUMP</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://blog.cloudflare.com/</t>
+          <t>https://dmpdump.github.io/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>DMPDUMP</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>https://dmpdump.github.io/</t>
+          <t>Forescout</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>https://www.forescout.com/blog</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Forescout</t>
+          <t>Genians</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>https://www.forescout.com/blog</t>
+          <t>https://www.genians.co.kr/en/blog/threat_intelligence</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Genians</t>
-        </is>
-      </c>
-      <c r="B123" s="7" t="inlineStr">
-        <is>
-          <t>https://www.genians.co.kr/en/blog/threat_intelligence</t>
+          <t>Koi Security</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://blog.koi.security/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Koi Security</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>https://blog.koi.security/</t>
+          <t>Oligo Security</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>https://www.oligo.security/blog/</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Oligo Security</t>
-        </is>
-      </c>
-      <c r="B125" s="7" t="inlineStr">
-        <is>
-          <t>https://www.oligo.security/blog/</t>
+          <t>Proofpoint</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://www.proofpoint.com/us/blog</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Phylum</t>
+          <t>QiAnXin XLab</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>https://blog.phylum.io/</t>
+          <t>https://blog.xlab.qianxin.com/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Proofpoint</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>https://www.proofpoint.com/us/blog</t>
+          <t>https://blog.qualys.com/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>QiAnXin XLab</t>
+          <t>QuickHeal</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>https://blog.xlab.qianxin.com/</t>
+          <t>https://blogs.quickheal.com</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Qualys</t>
+          <t>Rapid7</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>https://blog.qualys.com/</t>
+          <t>https://www.rapid7.com/blog/posts/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>QuickHeal</t>
+          <t>Recorded Future</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>https://blogs.quickheal.com</t>
+          <t>https://www.recordedfuture.com/blog
+https://www.recordedfuture.com/research/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Rapid7</t>
+          <t>Resecurity</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>https://www.rapid7.com/blog/posts/</t>
+          <t>https://www.resecurity.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Recorded Future</t>
+          <t>Reversing Labs</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>https://www.recordedfuture.com/blog
-https://www.recordedfuture.com/research/</t>
+          <t>https://www.reversinglabs.com/blog</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Resecurity</t>
+          <t>Rhino Security</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>https://www.resecurity.com/blog/</t>
+          <t>https://rhinosecuritylabs.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Reversing Labs</t>
+          <t>Salt Security</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>https://www.reversinglabs.com/blog</t>
+          <t>https://salt.security/blog/</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Rhino Security</t>
+          <t>SAM CERT</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>https://rhinosecuritylabs.com/blog/</t>
+          <t>https://www.samcert.gov.ws/samcert-advisories</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Salt Security</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>https://salt.security/blog/</t>
+          <t>Sectrio</t>
+        </is>
+      </c>
+      <c r="B136" s="8" t="inlineStr">
+        <is>
+          <t>https://sectrio.com/</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>SAM CERT</t>
+          <t>SecureList - Kaspersky</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>https://www.samcert.gov.ws/samcert-advisories</t>
+          <t>https://securelist.com/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Sectrio</t>
-        </is>
-      </c>
-      <c r="B138" s="8" t="inlineStr">
-        <is>
-          <t>https://sectrio.com/</t>
+          <t>Security Scorecard</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://securityscorecard.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>SecureList - Kaspersky</t>
+          <t>Securonix</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>https://securelist.com/</t>
+          <t>https://www.securonix.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Secureworks</t>
+          <t>Sekoia</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>https://www.secureworks.com/blog/</t>
+          <t>https://blog.sekoia.io/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Security Scorecard</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>https://securityscorecard.com/blog/</t>
+          <t>SentinelOne</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="inlineStr">
+        <is>
+          <t>https://www.sentinelone.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Securonix</t>
+          <t>Seqrite</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>https://www.securonix.com/blog/</t>
+          <t>https://www.seqrite.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Sekoia</t>
+          <t>Silent Push</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>https://blog.sekoia.io/</t>
+          <t>https://www.silentpush.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>SentinelOne</t>
-        </is>
-      </c>
-      <c r="B144" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sentinelone.com/blog/</t>
+          <t>Socket</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://socket.dev/blog/</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Seqrite</t>
+          <t>SOCradar</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>https://www.seqrite.com/blog/</t>
+          <t>https://socradar.io/blog/</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Silent Push</t>
+          <t>Sonar Source</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>https://www.silentpush.com/blog/</t>
+          <t>https://www.sonarsource.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Socket</t>
+          <t>Sonatype</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>https://socket.dev/blog/</t>
+          <t>https://www.sonatype.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>SOCradar</t>
+          <t>Sophos</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>https://socradar.io/blog/</t>
+          <t>https://news.sophos.com/en-us/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Sonar Source</t>
+          <t>SourceCode Red</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>https://www.sonarsource.com/blog/</t>
+          <t>https://sourcecodered.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Sonatype</t>
+          <t>Speartip</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>https://www.sonatype.com/blog/</t>
+          <t>https://www.speartip.com/resources/</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Sophos</t>
+          <t>Sucuri</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>https://news.sophos.com/en-us/</t>
+          <t>https://blog.sucuri.net/</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>SourceCode Red</t>
+          <t>Symantec - Broadcom</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>https://sourcecodered.com/blog/</t>
+          <t>https://www.security.com/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Speartip</t>
+          <t>Sysdig</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>https://www.speartip.com/resources/</t>
+          <t>https://sysdig.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Sucuri</t>
+          <t>Tenable</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>https://blog.sucuri.net/</t>
+          <t>https://www.tenable.com/blog</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Symantec - Broadcom</t>
+          <t>ThreatDown - Malwarebytes</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>https://www.security.com/</t>
+          <t>https://www.threatdown.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Sysdig</t>
+          <t>Top10VPN</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>https://sysdig.com/blog/</t>
+          <t>https://www.top10vpn.com/research/</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Tenable</t>
+          <t>Trellix</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>https://www.tenable.com/blog</t>
+          <t>https://www.trellix.com/blogs/research/
+https://www.trellix.com/blogs/</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>ThreatDown - Malwarebytes</t>
+          <t>Trend Micro</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>https://www.threatdown.com/blog/</t>
+          <t>https://www.trendmicro.com/en_us/research.html</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Top10VPN</t>
+          <t>TRM Labs</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>https://www.top10vpn.com/research/</t>
+          <t>https://www.trmlabs.com/resources/blog</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Trellix</t>
+          <t>Truffle Security</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>https://www.trellix.com/blogs/research/
-https://www.trellix.com/blogs/</t>
+          <t>https://trufflesecurity.com/blog</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Trend Micro</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>https://www.trendmicro.com/en_us/research.html</t>
+          <t>Trustwave</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
+        <is>
+          <t>https://www.trustwave.com/en-us/resources/blogs/spiderlabs-blog</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>TRM Labs</t>
+          <t>txOne</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>https://www.trmlabs.com/resources/blog</t>
+          <t>https://www.txone.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Truffle Security</t>
+          <t>Unit 42- Palo Alto Networks</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>https://trufflesecurity.com/blog</t>
+          <t>https://unit42.paloaltonetworks.com/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Trustwave</t>
-        </is>
-      </c>
-      <c r="B164" s="7" t="inlineStr">
-        <is>
-          <t>https://www.trustwave.com/en-us/resources/blogs/spiderlabs-blog</t>
+          <t>Uptycs</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://www.uptycs.com/blog</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>txOne</t>
+          <t>US Department of Justice</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>https://www.txone.com/blog/</t>
+          <t>https://www.justice.gov/</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Unit 42- Palo Alto Networks</t>
+          <t>US Treasury</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>https://unit42.paloaltonetworks.com/</t>
+          <t>https://home.treasury.gov/</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Uptycs</t>
+          <t>Validin</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>https://www.uptycs.com/blog</t>
+          <t>https://www.validin.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>US Department of Justice</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>https://www.justice.gov/</t>
+          <t>Varonis</t>
+        </is>
+      </c>
+      <c r="B168" s="7" t="inlineStr">
+        <is>
+          <t>https://www.varonis.com/blog</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>US Treasury</t>
+          <t>Virus Total</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>https://home.treasury.gov/</t>
+          <t>https://blog.virustotal.com/</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Validin</t>
+          <t>Vmware</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>https://www.validin.com/blog/</t>
+          <t>https://blogs.vmware.com/security/</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Varonis</t>
-        </is>
-      </c>
-      <c r="B171" s="7" t="inlineStr">
-        <is>
-          <t>https://www.varonis.com/blog</t>
+          <t>Volexity</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>https://www.volexity.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Veriti AI</t>
+          <t>WeLiveSecurity - ESET</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>https://veriti.ai/blog/veriti-research/</t>
+          <t>https://www.welivesecurity.com/en/</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Virus Total</t>
+          <t>Wiz</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>https://blog.virustotal.com/</t>
+          <t>https://www.wiz.io/blog/</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Vmware</t>
+          <t>Zimperium</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>https://blogs.vmware.com/security/</t>
+          <t>https://www.zimperium.com/blog</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Volexity</t>
+          <t>Zscaler</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>https://www.volexity.com/blog/</t>
+          <t>https://www.zscaler.com/blogs?type=security-research</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>WeLiveSecurity - ESET</t>
+          <t>Jamf</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>https://www.welivesecurity.com/en/</t>
+          <t>https://www.jamf.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>Wiz</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>https://www.wiz.io/blog/</t>
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Kroll</t>
+        </is>
+      </c>
+      <c r="B177" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kroll.com/en/</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Zimperium</t>
+          <t>StrongestLayer</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>https://www.zimperium.com/blog</t>
+          <t>https://www.strongestlayer.com/research</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Zscaler</t>
+          <t>LastPass</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>https://www.zscaler.com/blogs?type=security-research</t>
+          <t>https://blog.lastpass.com/</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>F6 Russia</t>
+          <t>Blackpoint</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>https://www.f6.ru/blog</t>
+          <t>https://blackpointcyber.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>Jamf</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>https://www.jamf.com/blog/</t>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Brave</t>
+        </is>
+      </c>
+      <c r="B181" s="7" t="inlineStr">
+        <is>
+          <t>https://brave.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>Kroll</t>
-        </is>
-      </c>
-      <c r="B182" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kroll.com/en/</t>
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Aryaka</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://www.aryaka.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="inlineStr">
-        <is>
-          <t>StrongestLayer</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>https://www.strongestlayer.com/research</t>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Sygnia</t>
+        </is>
+      </c>
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sygnia.co/blog/</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>LastPass</t>
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Schneier on Security</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>https://blog.lastpass.com/</t>
+          <t>https://www.schneier.com/feed/</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>Blackpoint</t>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Malware Traffic Analysis</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>https://blackpointcyber.com/blog/</t>
+          <t>https://www.malware-traffic-analysis.net/blog-entries.rss</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Brave</t>
-        </is>
-      </c>
-      <c r="B186" s="7" t="inlineStr">
-        <is>
-          <t>https://brave.com/blog/</t>
+          <t>VX-Underground</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://vx-underground.org/</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="inlineStr">
-        <is>
-          <t>Aryaka</t>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>SANS Internet Storm Center</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>https://www.aryaka.com/blog/</t>
+          <t>https://isc.sans.edu/rssfeed.xml</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Sygnia</t>
-        </is>
-      </c>
-      <c r="B188" s="7" t="inlineStr">
-        <is>
-          <t>https://www.sygnia.co/blog/</t>
+          <t>CERT-EU</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://cert.europa.eu/publications/threat-intelligence-rss</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Schneier on Security</t>
+          <t>Check Point Research (research.checkpoint.com)</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>https://www.schneier.com/feed/</t>
+          <t>https://research.checkpoint.com/feed/</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Malware Traffic Analysis</t>
+          <t>Snyk</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>https://www.malware-traffic-analysis.net/blog-entries.rss</t>
+          <t>https://snyk.io/blog/feed/</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>VX-Underground</t>
+          <t>GitHub Security Blog</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>https://vx-underground.org/</t>
+          <t>https://github.blog/security/feed/</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SANS Internet Storm Center</t>
+          <t>JFrog</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>https://isc.sans.edu/rssfeed.xml</t>
+          <t>https://jfrog.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CERT-EU</t>
+          <t>Wordfence</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>https://cert.europa.eu/publications/threat-intelligence-rss</t>
+          <t>https://www.wordfence.com/blog/feed/</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Check Point Research (research.checkpoint.com)</t>
+          <t>Orca Security</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>https://research.checkpoint.com/feed/</t>
+          <t>https://orca.security/resources/blog/feed/</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Snyk</t>
+          <t>Team Cymru</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>https://snyk.io/blog/feed/</t>
+          <t>https://www.team-cymru.com/post/rss.xml</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>GitHub Security Blog</t>
+          <t>Shadowserver</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>https://github.blog/security/feed/</t>
+          <t>https://www.shadowserver.org/news-insights/</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>JFrog</t>
+          <t>Cyble</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>https://jfrog.com/blog/</t>
+          <t>https://cyble.com/blog/feed/</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Wordfence</t>
+          <t>Anomali</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>https://www.wordfence.com/blog/feed/</t>
+          <t>https://www.anomali.com/blog</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Orca Security</t>
+          <t>NVISO</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>https://orca.security/resources/blog/feed/</t>
+          <t>https://blog.nviso.eu/feed/</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Team Cymru</t>
+          <t>Bishop Fox</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>https://www.team-cymru.com/post/rss.xml</t>
+          <t>https://bishopfox.com/feeds/blog.rss</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Shadowserver</t>
+          <t>Dragos</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>https://www.shadowserver.org/news-insights/</t>
+          <t>https://www.dragos.com/blog</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Cyble</t>
+          <t>SentinelOne Labs</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>https://cyble.com/blog/feed/</t>
+          <t>https://www.sentinelone.com/labs/feed/</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Anomali</t>
+          <t>CrowdSec</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>https://www.anomali.com/blog</t>
+          <t>https://www.crowdsec.net/blog/rss</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>NVISO</t>
+          <t>VMRay</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>https://blog.nviso.eu/feed/</t>
+          <t>https://www.vmray.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Bishop Fox</t>
+          <t>HarfangLab Coverage (via The Hacker News)</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>https://bishopfox.com/feeds/blog.rss</t>
+          <t>https://thehackernews.com/search?q=HarfangLab</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Dragos</t>
+          <t>Lab52 Coverage (via The Hacker News)</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>https://www.dragos.com/blog</t>
+          <t>https://thehackernews.com/search?q=Lab52</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>SentinelOne Labs</t>
+          <t>ACSC Coverage (via The Hacker News)</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>https://www.sentinelone.com/labs/feed/</t>
+          <t>https://thehackernews.com/search?q=ACSC</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>CrowdSec</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>https://www.crowdsec.net/blog/rss</t>
+          <t>https://arcticwolf.com/resources/blog/</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>VMRay</t>
+          <t>Check Point Research</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>https://www.vmray.com/blog/</t>
+          <t>https://blog.checkpoint.com/feed/</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>HarfangLab Coverage (via The Hacker News)</t>
+          <t>Check Point Exposure Management</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>https://thehackernews.com/search?q=HarfangLab</t>
+          <t>https://blog.checkpoint.com/exposure-management/feed/</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Lab52 Coverage (via The Hacker News)</t>
+          <t>Censys</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>https://thehackernews.com/search?q=Lab52</t>
+          <t>https://censys.com/feed/</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>ACSC Coverage (via The Hacker News)</t>
+          <t>PolySwarm</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>https://thehackernews.com/search?q=ACSC</t>
+          <t>https://blog.polyswarm.io/rss.xml</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Veracode</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>https://arcticwolf.com/resources/blog/</t>
+          <t>https://www.veracode.com/blog/</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Check Point Research</t>
+          <t>Zerobec</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>https://blog.checkpoint.com/feed/</t>
+          <t>https://zerobec.com/feed.xml</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Check Point Exposure Management</t>
+          <t>AISI</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>https://blog.checkpoint.com/exposure-management/feed/</t>
+          <t>https://www.aisi.gov.uk/blog/</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Censys</t>
+          <t>Manifold Security</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>https://censys.com/feed/</t>
+          <t>https://www.manifold.security/blog/</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>PolySwarm</t>
+          <t>Open Source Malware</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
-        <is>
-          <t>https://blog.polyswarm.io/rss.xml</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>Veracode</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>https://www.veracode.com/blog/</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>Zerobec</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>https://zerobec.com/feed.xml</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>AISI</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>https://www.aisi.gov.uk/blog/</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>Manifold Security</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>https://www.manifold.security/blog/</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>Open Source Malware</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
         <is>
           <t>https://opensourcemalware.com/rss.xml</t>
         </is>
@@ -3229,19 +3169,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" location="hub" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B166" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B173" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B184" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B188" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B166" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B173" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B184" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B188" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add TechCrunch Security as a CTI source
Uses the category RSS feed (techcrunch.com/category/security/feed/) --
clean, working, no bot protection, so type: feed rather than escalating
to a scraper. Pre-seeded state_seeds.json with the current 20 backlog
links so the first real run doesn't report them all as new.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CTI_Source_List.xlsx
+++ b/CTI_Source_List.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B217"/>
+  <dimension ref="A1:B218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="75" customWidth="1" style="4" min="1" max="1"/>
@@ -3108,6 +3108,18 @@
       <c r="B217" t="inlineStr">
         <is>
           <t>https://opensourcemalware.com/rss.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>TechCrunch Security</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/category/security/feed/</t>
         </is>
       </c>
     </row>

</xml_diff>